<commit_message>
data: stage coverage refresh 6/6
</commit_message>
<xml_diff>
--- a/diseases/d146/2010-2014.xlsx
+++ b/diseases/d146/2010-2014.xlsx
@@ -776,28 +776,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS2" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU2" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV2" t="inlineStr">
@@ -924,28 +938,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS3" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU3" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV3" t="inlineStr">
@@ -1072,28 +1100,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS4" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU4" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV4" t="inlineStr">
@@ -1220,28 +1262,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR5" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS5" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU5" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV5" t="inlineStr">
@@ -1368,28 +1424,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO6" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR6" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS6" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU6" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV6" t="inlineStr">
@@ -1516,28 +1586,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS7" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU7" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV7" t="inlineStr">
@@ -1664,28 +1748,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO8" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP8" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS8" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU8" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV8" t="inlineStr">
@@ -1812,28 +1910,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO9" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP9" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR9" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS9" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU9" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV9" t="inlineStr">
@@ -1960,28 +2072,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO10" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP10" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR10" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS10" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU10" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV10" t="inlineStr">
@@ -2108,28 +2234,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO11" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP11" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR11" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS11" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU11" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV11" t="inlineStr">
@@ -2256,28 +2396,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO12" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP12" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR12" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS12" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU12" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV12" t="inlineStr">
@@ -2404,28 +2558,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO13" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR13" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS13" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU13" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV13" t="inlineStr">
@@ -2552,28 +2720,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO14" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP14" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR14" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS14" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU14" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV14" t="inlineStr">
@@ -2700,28 +2882,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO15" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR15" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS15" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU15" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV15" t="inlineStr">
@@ -2848,28 +3044,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO16" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR16" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS16" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>HOLD_JP_0d0f562527f933882ae5ffa7bbb4</t>
+        </is>
+      </c>
       <c r="AT16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV16" t="inlineStr">

</xml_diff>